<commit_message>
Tested OpenCode. Goal was to compare it with Continue.dev. Made some fixes to Continue.dev report.
</commit_message>
<xml_diff>
--- a/project1/reports/continue.dev/comparison prompt 3.xlsx
+++ b/project1/reports/continue.dev/comparison prompt 3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\Project Bachelor\project 1 small\reports\continue.dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE6CA6A-4BA5-40BD-B3A7-F4D1A7788DD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB184EA5-AEAC-49F5-84CD-BC7E944D4FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1035" windowWidth="29040" windowHeight="15720" xr2:uid="{5C34DE08-A12C-4EAA-A114-EBB56ADF1C7F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5C34DE08-A12C-4EAA-A114-EBB56ADF1C7F}"/>
   </bookViews>
   <sheets>
     <sheet name="MyMath.checkSign(int)" sheetId="1" r:id="rId1"/>
@@ -1040,8 +1040,8 @@
       <c r="F7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>11</v>
+      <c r="G7" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>12</v>
@@ -1069,8 +1069,8 @@
       <c r="F8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>11</v>
+      <c r="G8" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>12</v>
@@ -2359,8 +2359,8 @@
       <c r="D10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>12</v>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>12</v>

</xml_diff>